<commit_message>
Add Batch E complaints tests: SR-064, SR-065, SR-068
3/3 passing on dev_namespaced_1:
- CFSUITE-SR-064 (CoM-Test-084) Create feedback/complaint requests for
  each sub-type (Comment, Complaint, Compliment) tagged via
  cfReq_Category.
- CFSUITE-SR-065 (CoM-Test-085) Complaint case linked to a parent
  request via ParentId; parent-child relationship queryable.
- CFSUITE-SR-068 (CoM-Test-088) Complaint case marked Confidential=Yes
  via API; field persists.

This org has no dedicated Complaint record type or picklist value, so
sub-type is recorded textually until a metadata-level complaint model
is introduced. Full sharing-rule verification (visibility scoped to a
complaint group) needs multi-user testing and is deferred.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Automated Testing CFSuite.xlsx
+++ b/documentation/Automated Testing CFSuite.xlsx
@@ -4721,6 +4721,11 @@
           <t>CFSUITE-SR-064</t>
         </is>
       </c>
+      <c r="AH102" s="47" t="inlineStr">
+        <is>
+          <t>CFSUITE-SR-064 (robot/tests/requests/CFSUITE-SR-064_create_feedback_and_complaint_requests.robot)</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="24" customHeight="1">
       <c r="A103" s="40" t="inlineStr">
@@ -4753,6 +4758,11 @@
       <c r="AG103" t="inlineStr">
         <is>
           <t>CFSUITE-SR-065</t>
+        </is>
+      </c>
+      <c r="AH103" s="47" t="inlineStr">
+        <is>
+          <t>CFSUITE-SR-065 (robot/tests/requests/CFSUITE-SR-065_create_complaint_as_child_of_request.robot)</t>
         </is>
       </c>
     </row>
@@ -4848,6 +4858,11 @@
       <c r="AG106" t="inlineStr">
         <is>
           <t>CFSUITE-SR-068</t>
+        </is>
+      </c>
+      <c r="AH106" s="47" t="inlineStr">
+        <is>
+          <t>CFSUITE-SR-068 (robot/tests/requests/CFSUITE-SR-068_restricted_access_to_complaints.robot)</t>
         </is>
       </c>
     </row>
@@ -9144,10 +9159,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH85" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH88" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH100" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH105" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH119" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH124" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH127" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH102" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH103" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH105" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH106" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH119" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH124" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH127" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>